<commit_message>
Add period cashflow appendix
</commit_message>
<xml_diff>
--- a/public/templates/cashflow/vvip-cashflow-corporate.xlsx
+++ b/public/templates/cashflow/vvip-cashflow-corporate.xlsx
@@ -6,14 +6,15 @@
   <sheets>
     <sheet sheetId="1" name="현금흐름표" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="업로드용_키값" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="작성가이드" state="visible" r:id="rId6"/>
+    <sheet sheetId="3" name="부록_기간별현금흐름" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="작성가이드" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="238">
   <si>
     <t>VVIP 법인 고객 현금흐름표</t>
   </si>
@@ -642,6 +643,51 @@
     <t>추가 상담 항목 1</t>
   </si>
   <si>
+    <t>부록 · 기간별 현금흐름</t>
+  </si>
+  <si>
+    <t>월별 유입·유출·저축/투자·세금 납부액을 입력하면 앱의 현금흐름 부록과 IPS 부록 표/차트에 반영됩니다. 금액 단위는 만원입니다.</t>
+  </si>
+  <si>
+    <t>기간(YYYY-MM)</t>
+  </si>
+  <si>
+    <t>유입(만원)</t>
+  </si>
+  <si>
+    <t>유출(만원)</t>
+  </si>
+  <si>
+    <t>저축/투자(만원)</t>
+  </si>
+  <si>
+    <t>세금납부(만원)</t>
+  </si>
+  <si>
+    <t>순현금흐름(만원)</t>
+  </si>
+  <si>
+    <t>누적순현금흐름(만원)</t>
+  </si>
+  <si>
+    <t>주요 이벤트/메모</t>
+  </si>
+  <si>
+    <t>정상 월간 현금흐름</t>
+  </si>
+  <si>
+    <t>세금 납부월 - 현금화 재원 확인</t>
+  </si>
+  <si>
+    <t>배당/상여 유입월</t>
+  </si>
+  <si>
+    <t>작성 원칙</t>
+  </si>
+  <si>
+    <t>앱은 앱 반영(Y/N)이 Y인 행만 읽습니다. 세금/회계 확정 판단이 아니라 상담용 추정이며 세무 전문가 확인이 필요합니다.</t>
+  </si>
+  <si>
     <t>가이드</t>
   </si>
   <si>
@@ -657,13 +703,19 @@
     <t>업로드 규칙</t>
   </si>
   <si>
-    <t>앱은 업로드용_키값 시트를 우선 읽고, 없으면 현금흐름표 본문에서 항목/금액 구조를 탐색합니다.</t>
+    <t>앱은 업로드용_키값 시트를 우선 읽고, 부록_기간별현금흐름 시트를 함께 읽어 현금흐름/IPS 부록 표와 차트에 반영합니다.</t>
   </si>
   <si>
     <t>앱 CashFlow 매핑</t>
   </si>
   <si>
     <t>항목→label, 값(만원)→amount, 납부일→date, 분류→category, 자금주체→entity, 계좌유형→accountType, 메모→taxAccountingNote</t>
+  </si>
+  <si>
+    <t>기간별 부록 매핑</t>
+  </si>
+  <si>
+    <t>기간→date, 유입/유출/저축/세금→amount, 주요 이벤트/메모→taxAccountingNote, 앱 반영(Y/N)→업로드 포함 여부</t>
   </si>
   <si>
     <t>세무·회계 유의</t>
@@ -682,7 +734,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -710,8 +762,13 @@
       <b/>
       <color rgb="FFFFFFFF"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FF111827"/>
+      <sz val="16"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -731,6 +788,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F2937"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3F4F6"/>
       </patternFill>
     </fill>
   </fills>
@@ -761,7 +823,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -788,6 +850,19 @@
     </xf>
     <xf numFmtId="3" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2796,7 +2871,467 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="3" width="14" style="8" customWidth="1"/>
+    <col min="4" max="4" width="16" style="8" customWidth="1"/>
+    <col min="5" max="5" width="14" style="8" customWidth="1"/>
+    <col min="6" max="6" width="18" style="8" customWidth="1"/>
+    <col min="7" max="7" width="20" style="8" customWidth="1"/>
+    <col min="8" max="8" width="34" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>209</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>210</v>
+      </c>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="10">
+        <v>46000</v>
+      </c>
+      <c r="C5" s="10">
+        <v>21000</v>
+      </c>
+      <c r="D5" s="10">
+        <v>15000</v>
+      </c>
+      <c r="E5" s="10">
+        <v>0</v>
+      </c>
+      <c r="F5" s="13">
+        <f>B5-C5-D5-E5</f>
+        <v>10000</v>
+      </c>
+      <c r="G5" s="13">
+        <f>F5</f>
+        <v>10000</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="B6" s="10">
+        <v>46000</v>
+      </c>
+      <c r="C6" s="10">
+        <v>21000</v>
+      </c>
+      <c r="D6" s="10">
+        <v>13000</v>
+      </c>
+      <c r="E6" s="10">
+        <v>0</v>
+      </c>
+      <c r="F6" s="13">
+        <f>B6-C6-D6-E6</f>
+        <v>12000</v>
+      </c>
+      <c r="G6" s="13">
+        <f>G5+F6</f>
+        <v>22000</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" s="10">
+        <v>46000</v>
+      </c>
+      <c r="C7" s="10">
+        <v>23000</v>
+      </c>
+      <c r="D7" s="10">
+        <v>13000</v>
+      </c>
+      <c r="E7" s="10">
+        <v>85000</v>
+      </c>
+      <c r="F7" s="13">
+        <f>B7-C7-D7-E7</f>
+        <v>-75000</v>
+      </c>
+      <c r="G7" s="13">
+        <f>G6+F7</f>
+        <v>-53000</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="B8" s="10">
+        <v>81000</v>
+      </c>
+      <c r="C8" s="10">
+        <v>21000</v>
+      </c>
+      <c r="D8" s="10">
+        <v>15000</v>
+      </c>
+      <c r="E8" s="10">
+        <v>0</v>
+      </c>
+      <c r="F8" s="13">
+        <f>B8-C8-D8-E8</f>
+        <v>45000</v>
+      </c>
+      <c r="G8" s="13">
+        <f>G7+F8</f>
+        <v>-8000</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="B9" s="10">
+        <v>46000</v>
+      </c>
+      <c r="C9" s="10">
+        <v>21000</v>
+      </c>
+      <c r="D9" s="10">
+        <v>13000</v>
+      </c>
+      <c r="E9" s="10">
+        <v>5200</v>
+      </c>
+      <c r="F9" s="13">
+        <f>B9-C9-D9-E9</f>
+        <v>6800</v>
+      </c>
+      <c r="G9" s="13">
+        <f>G8+F9</f>
+        <v>-1200</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="10">
+        <v>46000</v>
+      </c>
+      <c r="C10" s="10">
+        <v>21000</v>
+      </c>
+      <c r="D10" s="10">
+        <v>13000</v>
+      </c>
+      <c r="E10" s="10">
+        <v>0</v>
+      </c>
+      <c r="F10" s="13">
+        <f>B10-C10-D10-E10</f>
+        <v>12000</v>
+      </c>
+      <c r="G10" s="13">
+        <f>G9+F10</f>
+        <v>10800</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="B11" s="10">
+        <v>46000</v>
+      </c>
+      <c r="C11" s="10">
+        <v>21000</v>
+      </c>
+      <c r="D11" s="10">
+        <v>15000</v>
+      </c>
+      <c r="E11" s="10">
+        <v>900</v>
+      </c>
+      <c r="F11" s="13">
+        <f>B11-C11-D11-E11</f>
+        <v>9100</v>
+      </c>
+      <c r="G11" s="13">
+        <f>G10+F11</f>
+        <v>19900</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="B12" s="10">
+        <v>46000</v>
+      </c>
+      <c r="C12" s="10">
+        <v>22500</v>
+      </c>
+      <c r="D12" s="10">
+        <v>13000</v>
+      </c>
+      <c r="E12" s="10">
+        <v>0</v>
+      </c>
+      <c r="F12" s="13">
+        <f>B12-C12-D12-E12</f>
+        <v>10500</v>
+      </c>
+      <c r="G12" s="13">
+        <f>G11+F12</f>
+        <v>30400</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="10">
+        <v>46000</v>
+      </c>
+      <c r="C13" s="10">
+        <v>21000</v>
+      </c>
+      <c r="D13" s="10">
+        <v>13000</v>
+      </c>
+      <c r="E13" s="10">
+        <v>32000</v>
+      </c>
+      <c r="F13" s="13">
+        <f>B13-C13-D13-E13</f>
+        <v>-20000</v>
+      </c>
+      <c r="G13" s="13">
+        <f>G12+F13</f>
+        <v>10400</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B14" s="10">
+        <v>46000</v>
+      </c>
+      <c r="C14" s="10">
+        <v>21000</v>
+      </c>
+      <c r="D14" s="10">
+        <v>15000</v>
+      </c>
+      <c r="E14" s="10">
+        <v>0</v>
+      </c>
+      <c r="F14" s="13">
+        <f>B14-C14-D14-E14</f>
+        <v>10000</v>
+      </c>
+      <c r="G14" s="13">
+        <f>G13+F14</f>
+        <v>20400</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B15" s="10">
+        <v>46000</v>
+      </c>
+      <c r="C15" s="10">
+        <v>21000</v>
+      </c>
+      <c r="D15" s="10">
+        <v>13000</v>
+      </c>
+      <c r="E15" s="10">
+        <v>0</v>
+      </c>
+      <c r="F15" s="13">
+        <f>B15-C15-D15-E15</f>
+        <v>12000</v>
+      </c>
+      <c r="G15" s="13">
+        <f>G14+F15</f>
+        <v>32400</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="10">
+        <v>52000</v>
+      </c>
+      <c r="C16" s="10">
+        <v>21000</v>
+      </c>
+      <c r="D16" s="10">
+        <v>13000</v>
+      </c>
+      <c r="E16" s="10">
+        <v>12000</v>
+      </c>
+      <c r="F16" s="13">
+        <f>B16-C16-D16-E16</f>
+        <v>6000</v>
+      </c>
+      <c r="G16" s="13">
+        <f>G15+F16</f>
+        <v>38400</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="14" t="s">
+        <v>222</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>223</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -2808,12 +3343,12 @@
         <v>116</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>209</v>
+        <v>224</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>1</v>
@@ -2821,42 +3356,50 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>211</v>
+        <v>226</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>213</v>
+        <v>228</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>214</v>
+        <v>229</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>215</v>
+        <v>230</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>216</v>
+        <v>231</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>217</v>
+        <v>232</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>218</v>
+        <v>233</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>219</v>
+        <v>234</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>220</v>
+        <v>235</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>237</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix period cashflow tax line charts
</commit_message>
<xml_diff>
--- a/public/templates/cashflow/vvip-cashflow-corporate.xlsx
+++ b/public/templates/cashflow/vvip-cashflow-corporate.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="244">
   <si>
     <t>VVIP 법인 고객 현금흐름표</t>
   </si>
@@ -676,10 +676,28 @@
     <t>정상 월간 현금흐름</t>
   </si>
   <si>
-    <t>세금 납부월 - 현금화 재원 확인</t>
+    <t>법인세 납부월 - 현금화 재원 확인</t>
   </si>
   <si>
     <t>배당/상여 유입월</t>
+  </si>
+  <si>
+    <t>종합소득세 납부월 - 현금화 재원 확인</t>
+  </si>
+  <si>
+    <t>증여 실행 원금 유출월 - 증여세는 2026-09 반영</t>
+  </si>
+  <si>
+    <t>재산세 납부월 - 현금화 재원 확인</t>
+  </si>
+  <si>
+    <t>상속세 납부월 - 현금화 재원 확인</t>
+  </si>
+  <si>
+    <t>증여세 납부월 - 증여 실행 원금과 분리</t>
+  </si>
+  <si>
+    <t>법인 세금 예비월 - 단기 운용자금 확인</t>
   </si>
   <si>
     <t>작성 원칙</t>
@@ -3088,7 +3106,7 @@
         <v>-1200</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="I9" s="5" t="s">
         <v>62</v>
@@ -3102,7 +3120,7 @@
         <v>46000</v>
       </c>
       <c r="C10" s="10">
-        <v>21000</v>
+        <v>221000</v>
       </c>
       <c r="D10" s="10">
         <v>13000</v>
@@ -3112,14 +3130,14 @@
       </c>
       <c r="F10" s="13">
         <f>B10-C10-D10-E10</f>
-        <v>12000</v>
+        <v>-188000</v>
       </c>
       <c r="G10" s="13">
         <f>G9+F10</f>
-        <v>10800</v>
+        <v>-189200</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>62</v>
@@ -3147,10 +3165,10 @@
       </c>
       <c r="G11" s="13">
         <f>G10+F11</f>
-        <v>19900</v>
+        <v>-180100</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="I11" s="5" t="s">
         <v>62</v>
@@ -3170,18 +3188,18 @@
         <v>13000</v>
       </c>
       <c r="E12" s="10">
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="F12" s="13">
         <f>B12-C12-D12-E12</f>
-        <v>10500</v>
+        <v>-109500</v>
       </c>
       <c r="G12" s="13">
         <f>G11+F12</f>
-        <v>30400</v>
+        <v>-289600</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>62</v>
@@ -3209,10 +3227,10 @@
       </c>
       <c r="G13" s="13">
         <f>G12+F13</f>
-        <v>10400</v>
+        <v>-309600</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>62</v>
@@ -3240,7 +3258,7 @@
       </c>
       <c r="G14" s="13">
         <f>G13+F14</f>
-        <v>20400</v>
+        <v>-299600</v>
       </c>
       <c r="H14" s="5" t="s">
         <v>219</v>
@@ -3271,7 +3289,7 @@
       </c>
       <c r="G15" s="13">
         <f>G14+F15</f>
-        <v>32400</v>
+        <v>-287600</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>219</v>
@@ -3302,10 +3320,10 @@
       </c>
       <c r="G16" s="13">
         <f>G15+F16</f>
-        <v>38400</v>
+        <v>-281600</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>62</v>
@@ -3313,10 +3331,10 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -3343,12 +3361,12 @@
         <v>116</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>1</v>
@@ -3356,50 +3374,50 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>

</xml_diff>